<commit_message>
eliminados encuestas no validas
</commit_message>
<xml_diff>
--- a/Entrega final/Evaluación de Usabilidad AQuMaS - SUS Instrumento Base (respuestas) (1).xlsx
+++ b/Entrega final/Evaluación de Usabilidad AQuMaS - SUS Instrumento Base (respuestas) (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cris\Documents\GitHub\trabajo-de-grado-\Entrega final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0FFB4D6-D262-4BC9-AE72-9DF98E387B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23DDB6E-E7EE-4267-BA1E-2BA6CCC47196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Respuestas" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="175">
   <si>
     <t>Marca temporal</t>
   </si>
@@ -264,9 +264,6 @@
     <t>wilportilla225@umariana.edu.co</t>
   </si>
   <si>
-    <t>dansapuyes225@umariana.edu.co</t>
-  </si>
-  <si>
     <t>sheguzman225@umariana.edu.co</t>
   </si>
   <si>
@@ -276,15 +273,6 @@
     <t xml:space="preserve">Al momento de descargar los niveles mensuales y abrir el documento, debería estar ya organizado en tabla para no perder tiempo </t>
   </si>
   <si>
-    <t>brypastas225@umariana.edu.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es muy fácil de usar y comprender </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ninguno </t>
-  </si>
-  <si>
     <t>darosero225@umariana.edu.co</t>
   </si>
   <si>
@@ -297,18 +285,6 @@
     <t xml:space="preserve">Tutoriales o guias dentro de la aplicación </t>
   </si>
   <si>
-    <t>panirosero223@umariana.edu.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">muy organizado, la información se muestra clara, se puede descargar datos con facilidad y muy claros. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">En mi opinión, siento que el software está muy completo y listo para aplicarse </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ningunas, el uso de software es muy facil para manejar </t>
-  </si>
-  <si>
     <t>latapatino223@umariana.edu.co</t>
   </si>
   <si>
@@ -459,18 +435,6 @@
     <t>Interfaz simple, navegación clara, información resumida, carga rápida y opciones de personalización para el usuario.</t>
   </si>
   <si>
-    <t>ivmaperenguez123@umariana.edu.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los datos son claros, al momento de visualizarlos se puede identificarlos de manera adecuada y ordenada, además su sistema operativo en muy entendible </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Está bien estructurado </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un lenguaje hablado, como estilo servidor de siri, esto sería muy interesante </t>
-  </si>
-  <si>
     <t>maparosales123@umariana.edu.co</t>
   </si>
   <si>
@@ -483,18 +447,6 @@
     <t xml:space="preserve">Que se tenga en cuenta un posible prototipo el cual se coloque en mercado y ayude a otros lugares a conocer acerca de la calidad de aire y  generar datos </t>
   </si>
   <si>
-    <t>alexandra.piaguajeor212@umariana.edu.co</t>
-  </si>
-  <si>
-    <t>la facilidad de uso. Un buen software entenderlo y manejarlo sin necesidad de mucha explicación o capacitación.</t>
-  </si>
-  <si>
-    <t>rendimiento, logrando que el software sea más rápido, consuma menos recursos y no se bloquee o se vuelva lento.</t>
-  </si>
-  <si>
-    <t>También es clave incluir guías o tutoriales dentro del sistema, como instrucciones paso a paso, ayudas emergentes o asistentes que orienten al usuario al inicio.</t>
-  </si>
-  <si>
     <t>brdagarcia123@umariana.edu.co</t>
   </si>
   <si>
@@ -519,18 +471,6 @@
     <t xml:space="preserve">La batería también debería ser portátil que funcione en cualquier lugar donde se ubique </t>
   </si>
   <si>
-    <t>Jfaortega123@umariana.edu.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Tiene mucha innovación </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Hacerlo más portátil y que sea </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Que   puedan acceder sin ser estudiante  de la mariana </t>
-  </si>
-  <si>
     <t>mayeortega123@umariana.edu.co</t>
   </si>
   <si>
@@ -541,18 +481,6 @@
   </si>
   <si>
     <t>Me parece que esta muy fácil para acceder y usar, no tengo recomendaciones.</t>
-  </si>
-  <si>
-    <t>emsagarreta123@umariana.edu.co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es fácil de entender y fácil de manejar </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se tiene en cuenta otros contaminantes más peligrosos y también de acuerdo a la concentración de estos, se debería dar una recomendación por ejemplo si está muy alto una recomendación como más ventilación o algo parecido </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siento que es muy fácil de usar </t>
   </si>
   <si>
     <t>jcrodriguez222@umariana.edu.co</t>
@@ -1003,19 +931,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.41463414634146339</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.29268292682926828</c:v>
+                  <c:v>0.35294117647058826</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.3170731707317069E-2</c:v>
+                  <c:v>8.8235294117647065E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1951219512195122</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1271,19 +1199,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.24390243902439024</c:v>
+                  <c:v>0.29411764705882354</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.43902439024390244</c:v>
+                  <c:v>0.44117647058823528</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1951219512195122</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1586,55 +1514,55 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.3170731707317069E-2</c:v>
+                  <c:v>5.8823529411764705E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.12195121951219512</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1951219512195122</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.878048780487805E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.3170731707317069E-2</c:v>
+                  <c:v>8.8235294117647065E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.878048780487805E-2</c:v>
+                  <c:v>5.8823529411764705E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.878048780487805E-2</c:v>
+                  <c:v>5.8823529411764705E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1887,16 +1815,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.24390243902439024</c:v>
+                  <c:v>0.29411764705882354</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.65853658536585369</c:v>
+                  <c:v>0.61764705882352944</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.3170731707317069E-2</c:v>
+                  <c:v>5.8823529411764705E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2143,10 +2071,10 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.36585365853658536</c:v>
+                  <c:v>0.3235294117647059</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.63414634146341464</c:v>
+                  <c:v>0.67647058823529416</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2402,19 +2330,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1951219512195122</c:v>
+                  <c:v>0.23529411764705882</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.31707317073170732</c:v>
+                  <c:v>0.29411764705882354</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.43902439024390244</c:v>
+                  <c:v>0.41176470588235292</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2670,19 +2598,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.21951219512195122</c:v>
+                  <c:v>0.26470588235294118</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.14634146341463414</c:v>
+                  <c:v>0.17647058823529413</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.24390243902439024</c:v>
+                  <c:v>0.26470588235294118</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.21951219512195122</c:v>
+                  <c:v>0.14705882352941177</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.17073170731707318</c:v>
+                  <c:v>0.14705882352941177</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2938,19 +2866,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.878048780487805E-2</c:v>
+                  <c:v>5.8823529411764705E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.17073170731707318</c:v>
+                  <c:v>0.20588235294117646</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.3170731707317069E-2</c:v>
+                  <c:v>8.8235294117647065E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.36585365853658536</c:v>
+                  <c:v>0.35294117647058826</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.34146341463414637</c:v>
+                  <c:v>0.29411764705882354</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3206,19 +3134,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.48780487804878048</c:v>
+                  <c:v>0.58823529411764708</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.21951219512195122</c:v>
+                  <c:v>0.26470588235294118</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.17073170731707318</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3474,19 +3402,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14634146341463414</c:v>
+                  <c:v>0.17647058823529413</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.41463414634146339</c:v>
+                  <c:v>0.41176470588235292</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3902439024390244</c:v>
+                  <c:v>0.35294117647058826</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3742,19 +3670,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.43902439024390244</c:v>
+                  <c:v>0.52941176470588236</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.26829268292682928</c:v>
+                  <c:v>0.3235294117647059</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.17073170731707318</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4010,19 +3938,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.4390243902439025E-2</c:v>
+                  <c:v>2.9411764705882353E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.878048780487805E-2</c:v>
+                  <c:v>5.8823529411764705E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.56097560975609762</c:v>
+                  <c:v>0.58823529411764708</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.26829268292682928</c:v>
+                  <c:v>0.20588235294117646</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4278,19 +4206,19 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.41463414634146339</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.1951219512195122</c:v>
+                  <c:v>0.23529411764705882</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.14634146341463414</c:v>
+                  <c:v>0.17647058823529413</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.14634146341463414</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>8.8235294117647065E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12018,7 +11946,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:S42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:S35">
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Marca temporal"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Dirección de correo electrónico"/>
@@ -12245,7 +12173,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
@@ -12279,34 +12207,34 @@
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>176</v>
+        <v>152</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>177</v>
+        <v>153</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>178</v>
+        <v>154</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>179</v>
+        <v>155</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>181</v>
+        <v>157</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>182</v>
+        <v>158</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>183</v>
+        <v>159</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>6</v>
@@ -13081,7 +13009,7 @@
     </row>
     <row r="15" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>46122.571542199075</v>
+        <v>46122.571666087963</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>69</v>
@@ -13099,51 +13027,57 @@
         <v>56</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="M15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="P15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N15" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
+      <c r="Q15" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="R15" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="S15" s="3" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="16" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>46122.571666087963</v>
+        <v>46122.586143645836</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C16" s="3">
         <v>18</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>55</v>
@@ -13152,175 +13086,171 @@
         <v>56</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="M16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="N16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="O16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="O16" s="3" t="s">
+      <c r="P16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P16" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="Q16" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R16" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>46122.572836354171</v>
+        <v>46122.687465358795</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C17" s="3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>56</v>
       </c>
       <c r="G17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>16</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>16</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>16</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>16</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="R17" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="S17" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>46122.586143645836</v>
+        <v>46122.697414699069</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C18" s="3">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="J18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J18" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="K18" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q18" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="R18" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="S18" s="3" t="s">
-        <v>79</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
     </row>
     <row r="19" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>46122.684534641201</v>
+        <v>46122.699353761578</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C19" s="3">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>55</v>
@@ -13329,81 +13259,81 @@
         <v>56</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K19" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J19" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="L19" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>22</v>
       </c>
       <c r="O19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="P19" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="P19" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="Q19" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>46122.687465358795</v>
+        <v>46122.699506307872</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C20" s="3">
         <v>23</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>56</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>13</v>
@@ -13412,48 +13342,48 @@
         <v>16</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P20" s="3" t="s">
         <v>16</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>46122.697414699069</v>
+        <v>46122.708347662032</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C21" s="3">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>16</v>
@@ -13477,23 +13407,27 @@
         <v>16</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="R21" s="3"/>
-      <c r="S21" s="3"/>
+        <v>93</v>
+      </c>
+      <c r="R21" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="S21" s="3" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="22" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>46122.699353761578</v>
+        <v>46122.70842112269</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C22" s="3">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>55</v>
@@ -13502,81 +13436,81 @@
         <v>56</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>15</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P22" s="3" t="s">
         <v>16</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>46122.699506307872</v>
+        <v>46125.40491892361</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C23" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>56</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M23" s="3" t="s">
         <v>13</v>
@@ -13588,27 +13522,25 @@
         <v>14</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="S23" s="3" t="s">
-        <v>99</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="S23" s="3"/>
     </row>
     <row r="24" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>46122.708347662032</v>
+        <v>46125.405235011574</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C24" s="3">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>21</v>
@@ -13623,13 +13555,13 @@
         <v>13</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>13</v>
@@ -13638,7 +13570,7 @@
         <v>16</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>16</v>
@@ -13647,27 +13579,27 @@
         <v>13</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>46122.70842112269</v>
+        <v>46125.405716435183</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C25" s="3">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>21</v>
@@ -13679,13 +13611,13 @@
         <v>56</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>22</v>
@@ -13697,39 +13629,37 @@
         <v>22</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="O25" s="3" t="s">
         <v>13</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="S25" s="3" t="s">
-        <v>107</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="S25" s="3"/>
     </row>
     <row r="26" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>46125.40491892361</v>
+        <v>46125.406938287037</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C26" s="3">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>55</v>
@@ -13738,49 +13668,51 @@
         <v>56</v>
       </c>
       <c r="G26" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H26" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="I26" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="J26" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L26" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K26" s="3" t="s">
+      <c r="M26" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="N26" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L26" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M26" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="N26" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="O26" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P26" s="3" t="s">
         <v>22</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="S26" s="3"/>
+        <v>112</v>
+      </c>
+      <c r="S26" s="3" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="27" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>46125.405235011574</v>
+        <v>46125.406971354168</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C27" s="3">
         <v>20</v>
@@ -13798,13 +13730,13 @@
         <v>13</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="K27" s="3" t="s">
         <v>13</v>
@@ -13813,36 +13745,36 @@
         <v>16</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="O27" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P27" s="3" t="s">
         <v>14</v>
       </c>
       <c r="Q27" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="R27" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="S27" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>46125.405716435183</v>
+        <v>46125.407009629635</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C28" s="3">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>21</v>
@@ -13854,13 +13786,13 @@
         <v>56</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>22</v>
@@ -13884,25 +13816,27 @@
         <v>14</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="S28" s="3"/>
+        <v>120</v>
+      </c>
+      <c r="S28" s="3" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="29" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>46125.406938287037</v>
+        <v>46125.407198715278</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C29" s="3">
+        <v>22</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>55</v>
@@ -13911,54 +13845,54 @@
         <v>56</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H29" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I29" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="K29" s="3" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="L29" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M29" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M29" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="N29" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>46125.406971354168</v>
+        <v>46125.407518472217</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C30" s="3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>21</v>
@@ -13976,10 +13910,10 @@
         <v>22</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="K30" s="3" t="s">
         <v>13</v>
@@ -13988,39 +13922,39 @@
         <v>16</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>46125.407009629635</v>
+        <v>46125.407928287037</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C31" s="3">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>55</v>
@@ -14029,19 +13963,19 @@
         <v>56</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>22</v>
@@ -14053,92 +13987,92 @@
         <v>22</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>46125.407198715278</v>
+        <v>46125.408008090279</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C32" s="3">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>56</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I32" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M32" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="J32" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K32" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L32" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="M32" s="3" t="s">
-        <v>13</v>
       </c>
       <c r="N32" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="P32" s="3" t="s">
         <v>14</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>46125.407317881945</v>
+        <v>46125.408516388889</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C33" s="3">
         <v>21</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>55</v>
@@ -14147,54 +14081,54 @@
         <v>56</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>46125.407518472217</v>
+        <v>46125.409171527775</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C34" s="3">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>21</v>
@@ -14206,57 +14140,57 @@
         <v>56</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M34" s="3" t="s">
         <v>13</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>46125.407539097221</v>
+        <v>46125.428013067125</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C35" s="3">
         <v>21</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>55</v>
@@ -14265,456 +14199,43 @@
         <v>56</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="36" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="2">
-        <v>46125.407928287037</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C36" s="3">
-        <v>25</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K36" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M36" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="N36" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="O36" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="P36" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q36" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="R36" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="S36" s="3" t="s">
         <v>149</v>
-      </c>
-    </row>
-    <row r="37" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="2">
-        <v>46125.408008090279</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="C37" s="3">
-        <v>25</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K37" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M37" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="N37" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O37" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="P37" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q37" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="R37" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="S37" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="2">
-        <v>46125.408134976853</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="C38" s="3">
-        <v>21</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M38" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="O38" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="P38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q38" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="R38" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="S38" s="3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="2">
-        <v>46125.408516388889</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C39" s="3">
-        <v>21</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G39" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K39" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L39" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M39" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="N39" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="O39" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P39" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q39" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="R39" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="S39" s="3" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="40" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="2">
-        <v>46125.408636840279</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C40" s="3">
-        <v>21</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K40" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L40" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M40" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="N40" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="O40" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="P40" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q40" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="R40" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="S40" s="3" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="41" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="2">
-        <v>46125.409171527775</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C41" s="3">
-        <v>23</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K41" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="M41" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="N41" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O41" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="P41" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q41" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="R41" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="S41" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="42" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="2">
-        <v>46125.428013067125</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="C42" s="3">
-        <v>21</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J42" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K42" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="L42" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="M42" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="N42" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="O42" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P42" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q42" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="R42" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="S42" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -14737,13 +14258,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -14751,12 +14272,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$O$2:$O$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$O$2:$O$35,"="&amp;A2)</f>
         <v>17</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>0.41463414634146339</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -14764,12 +14285,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$O$2:$O$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$O$2:$O$35,"="&amp;A3)</f>
         <v>8</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>0.1951219512195122</v>
+        <v>0.23529411764705882</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -14777,12 +14298,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$O$2:$O$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$O$2:$O$35,"="&amp;A4)</f>
         <v>6</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>0.14634146341463414</v>
+        <v>0.17647058823529413</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -14790,12 +14311,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$O$2:$O$42,"="&amp;A5)</f>
-        <v>6</v>
+        <f>COUNTIFS(Respuestas!$O$2:$O$35,"="&amp;A5)</f>
+        <v>0</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.14634146341463414</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -14803,21 +14324,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$O$2:$O$42,"="&amp;A6)</f>
-        <v>4</v>
+        <f>COUNTIFS(Respuestas!$O$2:$O$35,"="&amp;A6)</f>
+        <v>3</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>9.7560975609756101E-2</v>
+        <v>8.8235294117647065E-2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -14826,11 +14347,11 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="C9" s="8">
         <f>C2+C3</f>
-        <v>0.6097560975609756</v>
+        <v>0.73529411764705888</v>
       </c>
     </row>
   </sheetData>
@@ -14850,13 +14371,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
-        <v>197</v>
+        <v>173</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -14864,12 +14385,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$P$2:$P$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$P$2:$P$35,"="&amp;A2)</f>
         <v>1</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -14877,12 +14398,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$P$2:$P$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$P$2:$P$35,"="&amp;A3)</f>
         <v>4</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>9.7560975609756101E-2</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -14890,12 +14411,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$P$2:$P$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$P$2:$P$35,"="&amp;A4)</f>
         <v>10</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>0.24390243902439024</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -14903,12 +14424,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$P$2:$P$42,"="&amp;A5)</f>
-        <v>18</v>
+        <f>COUNTIFS(Respuestas!$P$2:$P$35,"="&amp;A5)</f>
+        <v>15</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.43902439024390244</v>
+        <v>0.44117647058823528</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -14916,21 +14437,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$P$2:$P$42,"="&amp;A6)</f>
-        <v>8</v>
+        <f>COUNTIFS(Respuestas!$P$2:$P$35,"="&amp;A6)</f>
+        <v>4</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>0.1951219512195122</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -14967,10 +14488,10 @@
         <v>2</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -14978,12 +14499,12 @@
         <v>17</v>
       </c>
       <c r="B2" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A2)</f>
         <v>1</v>
       </c>
       <c r="C2" s="19">
         <f>B2/$B$19</f>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -14991,12 +14512,12 @@
         <v>18</v>
       </c>
       <c r="B3" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A3)</f>
-        <v>3</v>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A3)</f>
+        <v>2</v>
       </c>
       <c r="C3" s="19">
         <f t="shared" ref="C3:C18" si="0">B3/$B$19</f>
-        <v>7.3170731707317069E-2</v>
+        <v>5.8823529411764705E-2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -15004,12 +14525,12 @@
         <v>19</v>
       </c>
       <c r="B4" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A4)</f>
         <v>4</v>
       </c>
       <c r="C4" s="19">
         <f t="shared" si="0"/>
-        <v>9.7560975609756101E-2</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -15017,12 +14538,12 @@
         <v>20</v>
       </c>
       <c r="B5" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A5)</f>
-        <v>5</v>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A5)</f>
+        <v>4</v>
       </c>
       <c r="C5" s="19">
         <f t="shared" si="0"/>
-        <v>0.12195121951219512</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -15030,12 +14551,12 @@
         <v>21</v>
       </c>
       <c r="B6" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A6)</f>
-        <v>8</v>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A6)</f>
+        <v>4</v>
       </c>
       <c r="C6" s="19">
         <f t="shared" si="0"/>
-        <v>0.1951219512195122</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -15043,12 +14564,12 @@
         <v>22</v>
       </c>
       <c r="B7" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A7)</f>
-        <v>2</v>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A7)</f>
+        <v>1</v>
       </c>
       <c r="C7" s="19">
         <f t="shared" si="0"/>
-        <v>4.878048780487805E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -15056,12 +14577,12 @@
         <v>23</v>
       </c>
       <c r="B8" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A8)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="19">
         <f t="shared" si="0"/>
-        <v>9.7560975609756101E-2</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -15069,12 +14590,12 @@
         <v>25</v>
       </c>
       <c r="B9" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A9)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A9)</f>
         <v>3</v>
       </c>
       <c r="C9" s="19">
         <f t="shared" si="0"/>
-        <v>7.3170731707317069E-2</v>
+        <v>8.8235294117647065E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -15082,12 +14603,12 @@
         <v>27</v>
       </c>
       <c r="B10" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A10)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A10)</f>
         <v>1</v>
       </c>
       <c r="C10" s="19">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -15095,12 +14616,12 @@
         <v>28</v>
       </c>
       <c r="B11" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A11)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A11)</f>
         <v>1</v>
       </c>
       <c r="C11" s="19">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -15108,12 +14629,12 @@
         <v>35</v>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A12)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A12)</f>
         <v>1</v>
       </c>
       <c r="C12" s="19">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -15121,12 +14642,12 @@
         <v>38</v>
       </c>
       <c r="B13" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A13)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A13)</f>
         <v>2</v>
       </c>
       <c r="C13" s="19">
         <f t="shared" si="0"/>
-        <v>4.878048780487805E-2</v>
+        <v>5.8823529411764705E-2</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -15134,12 +14655,12 @@
         <v>39</v>
       </c>
       <c r="B14" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A14)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A14)</f>
         <v>1</v>
       </c>
       <c r="C14" s="19">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -15147,12 +14668,12 @@
         <v>43</v>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A15)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A15)</f>
         <v>1</v>
       </c>
       <c r="C15" s="19">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -15160,12 +14681,12 @@
         <v>46</v>
       </c>
       <c r="B16" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A16)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A16)</f>
         <v>1</v>
       </c>
       <c r="C16" s="19">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -15173,12 +14694,12 @@
         <v>49</v>
       </c>
       <c r="B17" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A17)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A17)</f>
         <v>2</v>
       </c>
       <c r="C17" s="19">
         <f t="shared" si="0"/>
-        <v>4.878048780487805E-2</v>
+        <v>5.8823529411764705E-2</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -15186,25 +14707,25 @@
         <v>53</v>
       </c>
       <c r="B18" s="18">
-        <f>COUNTIFS(Respuestas!$C$2:$C$42,"="&amp;A18)</f>
+        <f>COUNTIFS(Respuestas!$C$2:$C$35,"="&amp;A18)</f>
         <v>1</v>
       </c>
       <c r="C18" s="19">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="B19">
         <f>SUM(B2:B18)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C19" s="20">
         <f>SUM(C2:C18)</f>
-        <v>1.0000000000000002</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -15231,10 +14752,10 @@
         <v>4</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -15242,12 +14763,12 @@
         <v>11</v>
       </c>
       <c r="B2" s="18">
-        <f>COUNTIFS(Respuestas!$E$2:$E$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$E$2:$E$35,"="&amp;A2)</f>
         <v>10</v>
       </c>
       <c r="C2" s="23">
         <f>B2/$B$6</f>
-        <v>0.24390243902439024</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15255,47 +14776,47 @@
         <v>55</v>
       </c>
       <c r="B3" s="18">
-        <f>COUNTIFS(Respuestas!$E$2:$E$42,"="&amp;A3)</f>
-        <v>27</v>
+        <f>COUNTIFS(Respuestas!$E$2:$E$35,"="&amp;A3)</f>
+        <v>21</v>
       </c>
       <c r="C3" s="23">
         <f t="shared" ref="C3:C5" si="0">B3/$B$6</f>
-        <v>0.65853658536585369</v>
+        <v>0.61764705882352944</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B4" s="18">
-        <f>COUNTIFS(Respuestas!$E$2:$E$42,"="&amp;A4)</f>
-        <v>3</v>
+        <f>COUNTIFS(Respuestas!$E$2:$E$35,"="&amp;A4)</f>
+        <v>2</v>
       </c>
       <c r="C4" s="23">
         <f t="shared" si="0"/>
-        <v>7.3170731707317069E-2</v>
+        <v>5.8823529411764705E-2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B5" s="18">
-        <f>COUNTIFS(Respuestas!$E$2:$E$42,"="&amp;A5)</f>
+        <f>COUNTIFS(Respuestas!$E$2:$E$35,"="&amp;A5)</f>
         <v>1</v>
       </c>
       <c r="C5" s="23">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="B6">
         <f>SUM(B2:B5)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C6" s="22">
         <f>SUM(C2:C5)</f>
@@ -15323,10 +14844,10 @@
         <v>3</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -15334,12 +14855,12 @@
         <v>10</v>
       </c>
       <c r="B2" s="18">
-        <f>COUNTIFS(Respuestas!$D$2:$D$42,"="&amp;A2)</f>
-        <v>15</v>
+        <f>COUNTIFS(Respuestas!$D$2:$D$35,"="&amp;A2)</f>
+        <v>11</v>
       </c>
       <c r="C2" s="23">
         <f>B2/$B$4</f>
-        <v>0.36585365853658536</v>
+        <v>0.3235294117647059</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15347,21 +14868,21 @@
         <v>21</v>
       </c>
       <c r="B3" s="18">
-        <f>COUNTIFS(Respuestas!$D$2:$D$42,"="&amp;A3)</f>
-        <v>26</v>
+        <f>COUNTIFS(Respuestas!$D$2:$D$35,"="&amp;A3)</f>
+        <v>23</v>
       </c>
       <c r="C3" s="23">
         <f>B3/$B$4</f>
-        <v>0.63414634146341464</v>
+        <v>0.67647058823529416</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="B4">
         <f>SUM(B2:B3)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C4" s="22">
         <f>SUM(C2:C3)</f>
@@ -15386,13 +14907,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -15400,12 +14921,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$G$2:$G$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$G$2:$G$35,"="&amp;A2)</f>
         <v>17</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>0.41463414634146339</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15413,12 +14934,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$G$2:$G$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$G$2:$G$35,"="&amp;A3)</f>
         <v>12</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>0.29268292682926828</v>
+        <v>0.35294117647058826</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -15426,12 +14947,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$G$2:$G$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$G$2:$G$35,"="&amp;A4)</f>
         <v>3</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>7.3170731707317069E-2</v>
+        <v>8.8235294117647065E-2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -15439,12 +14960,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$G$2:$G$42,"="&amp;A5)</f>
-        <v>8</v>
+        <f>COUNTIFS(Respuestas!$G$2:$G$35,"="&amp;A5)</f>
+        <v>1</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.1951219512195122</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -15452,21 +14973,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$G$2:$G$42,"="&amp;A6)</f>
+        <f>COUNTIFS(Respuestas!$G$2:$G$35,"="&amp;A6)</f>
         <v>1</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -15475,11 +14996,11 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="C9" s="8">
         <f>C2+C3</f>
-        <v>0.70731707317073167</v>
+        <v>0.85294117647058831</v>
       </c>
     </row>
   </sheetData>
@@ -15499,13 +15020,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -15513,12 +15034,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$H$2:$H$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$H$2:$H$35,"="&amp;A2)</f>
         <v>1</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15526,12 +15047,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$H$2:$H$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$H$2:$H$35,"="&amp;A3)</f>
         <v>1</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -15539,12 +15060,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$H$2:$H$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$H$2:$H$35,"="&amp;A4)</f>
         <v>8</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>0.1951219512195122</v>
+        <v>0.23529411764705882</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -15552,12 +15073,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$H$2:$H$42,"="&amp;A5)</f>
-        <v>13</v>
+        <f>COUNTIFS(Respuestas!$H$2:$H$35,"="&amp;A5)</f>
+        <v>10</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.31707317073170732</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -15565,21 +15086,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$H$2:$H$42,"="&amp;A6)</f>
-        <v>18</v>
+        <f>COUNTIFS(Respuestas!$H$2:$H$35,"="&amp;A6)</f>
+        <v>14</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>0.43902439024390244</v>
+        <v>0.41176470588235292</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -15613,13 +15134,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>190</v>
+        <v>166</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -15627,12 +15148,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$I$2:$I$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$I$2:$I$35,"="&amp;A2)</f>
         <v>9</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>0.21951219512195122</v>
+        <v>0.26470588235294118</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15640,12 +15161,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$I$2:$I$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$I$2:$I$35,"="&amp;A3)</f>
         <v>6</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>0.14634146341463414</v>
+        <v>0.17647058823529413</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -15653,12 +15174,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$I$2:$I$42,"="&amp;A4)</f>
-        <v>10</v>
+        <f>COUNTIFS(Respuestas!$I$2:$I$35,"="&amp;A4)</f>
+        <v>9</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>0.24390243902439024</v>
+        <v>0.26470588235294118</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -15666,12 +15187,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$I$2:$I$42,"="&amp;A5)</f>
-        <v>9</v>
+        <f>COUNTIFS(Respuestas!$I$2:$I$35,"="&amp;A5)</f>
+        <v>5</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.21951219512195122</v>
+        <v>0.14705882352941177</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -15679,21 +15200,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$I$2:$I$42,"="&amp;A6)</f>
-        <v>7</v>
+        <f>COUNTIFS(Respuestas!$I$2:$I$35,"="&amp;A6)</f>
+        <v>5</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>0.17073170731707318</v>
+        <v>0.14705882352941177</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -15702,11 +15223,11 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="C9" s="8">
         <f>C2+C3</f>
-        <v>0.36585365853658536</v>
+        <v>0.44117647058823528</v>
       </c>
     </row>
   </sheetData>
@@ -15726,13 +15247,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -15740,12 +15261,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$J$2:$J$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$J$2:$J$35,"="&amp;A2)</f>
         <v>2</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>4.878048780487805E-2</v>
+        <v>5.8823529411764705E-2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15753,12 +15274,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$J$2:$J$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$J$2:$J$35,"="&amp;A3)</f>
         <v>7</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>0.17073170731707318</v>
+        <v>0.20588235294117646</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -15766,12 +15287,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$J$2:$J$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$J$2:$J$35,"="&amp;A4)</f>
         <v>3</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>7.3170731707317069E-2</v>
+        <v>8.8235294117647065E-2</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -15779,12 +15300,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$J$2:$J$42,"="&amp;A5)</f>
-        <v>15</v>
+        <f>COUNTIFS(Respuestas!$J$2:$J$35,"="&amp;A5)</f>
+        <v>12</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.36585365853658536</v>
+        <v>0.35294117647058826</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -15792,21 +15313,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$J$2:$J$42,"="&amp;A6)</f>
-        <v>14</v>
+        <f>COUNTIFS(Respuestas!$J$2:$J$35,"="&amp;A6)</f>
+        <v>10</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>0.34146341463414637</v>
+        <v>0.29411764705882354</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -15840,13 +15361,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -15854,12 +15375,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$K$2:$K$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$K$2:$K$35,"="&amp;A2)</f>
         <v>20</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>0.48780487804878048</v>
+        <v>0.58823529411764708</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15867,12 +15388,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$K$2:$K$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$K$2:$K$35,"="&amp;A3)</f>
         <v>9</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>0.21951219512195122</v>
+        <v>0.26470588235294118</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -15880,12 +15401,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$K$2:$K$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$K$2:$K$35,"="&amp;A4)</f>
         <v>4</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>9.7560975609756101E-2</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -15893,12 +15414,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$K$2:$K$42,"="&amp;A5)</f>
-        <v>7</v>
+        <f>COUNTIFS(Respuestas!$K$2:$K$35,"="&amp;A5)</f>
+        <v>0</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.17073170731707318</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -15906,21 +15427,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$K$2:$K$42,"="&amp;A6)</f>
+        <f>COUNTIFS(Respuestas!$K$2:$K$35,"="&amp;A6)</f>
         <v>1</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -15929,11 +15450,11 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="C9" s="8">
         <f>C2+C3</f>
-        <v>0.70731707317073167</v>
+        <v>0.85294117647058831</v>
       </c>
     </row>
   </sheetData>
@@ -15953,13 +15474,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -15967,12 +15488,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$L$2:$L$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$L$2:$L$35,"="&amp;A2)</f>
         <v>1</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -15980,12 +15501,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$L$2:$L$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$L$2:$L$35,"="&amp;A3)</f>
         <v>1</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -15993,12 +15514,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$L$2:$L$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$L$2:$L$35,"="&amp;A4)</f>
         <v>6</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>0.14634146341463414</v>
+        <v>0.17647058823529413</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -16006,12 +15527,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$L$2:$L$42,"="&amp;A5)</f>
-        <v>17</v>
+        <f>COUNTIFS(Respuestas!$L$2:$L$35,"="&amp;A5)</f>
+        <v>14</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.41463414634146339</v>
+        <v>0.41176470588235292</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -16019,21 +15540,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$L$2:$L$42,"="&amp;A6)</f>
-        <v>16</v>
+        <f>COUNTIFS(Respuestas!$L$2:$L$35,"="&amp;A6)</f>
+        <v>12</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>0.3902439024390244</v>
+        <v>0.35294117647058826</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -16067,13 +15588,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -16081,12 +15602,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$M$2:$M$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$M$2:$M$35,"="&amp;A2)</f>
         <v>18</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>0.43902439024390244</v>
+        <v>0.52941176470588236</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -16094,12 +15615,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$M$2:$M$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$M$2:$M$35,"="&amp;A3)</f>
         <v>11</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>0.26829268292682928</v>
+        <v>0.3235294117647059</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -16107,12 +15628,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$M$2:$M$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$M$2:$M$35,"="&amp;A4)</f>
         <v>4</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>9.7560975609756101E-2</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -16120,12 +15641,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$M$2:$M$42,"="&amp;A5)</f>
-        <v>7</v>
+        <f>COUNTIFS(Respuestas!$M$2:$M$35,"="&amp;A5)</f>
+        <v>1</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.17073170731707318</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -16133,21 +15654,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$M$2:$M$42,"="&amp;A6)</f>
-        <v>1</v>
+        <f>COUNTIFS(Respuestas!$M$2:$M$35,"="&amp;A6)</f>
+        <v>0</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>2.4390243902439025E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
@@ -16156,11 +15677,11 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="C9" s="8">
         <f>C2+C3</f>
-        <v>0.70731707317073167</v>
+        <v>0.85294117647058831</v>
       </c>
     </row>
   </sheetData>
@@ -16180,13 +15701,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -16194,12 +15715,12 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <f>COUNTIFS(Respuestas!$N$2:$N$42,"="&amp;A2)</f>
+        <f>COUNTIFS(Respuestas!$N$2:$N$35,"="&amp;A2)</f>
         <v>1</v>
       </c>
       <c r="C2" s="8">
         <f>B2/$B$7</f>
-        <v>2.4390243902439025E-2</v>
+        <v>2.9411764705882353E-2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -16207,12 +15728,12 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <f>COUNTIFS(Respuestas!$N$2:$N$42,"="&amp;A3)</f>
+        <f>COUNTIFS(Respuestas!$N$2:$N$35,"="&amp;A3)</f>
         <v>2</v>
       </c>
       <c r="C3" s="8">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7</f>
-        <v>4.878048780487805E-2</v>
+        <v>5.8823529411764705E-2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -16220,12 +15741,12 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <f>COUNTIFS(Respuestas!$N$2:$N$42,"="&amp;A4)</f>
+        <f>COUNTIFS(Respuestas!$N$2:$N$35,"="&amp;A4)</f>
         <v>4</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>9.7560975609756101E-2</v>
+        <v>0.11764705882352941</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
@@ -16233,12 +15754,12 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <f>COUNTIFS(Respuestas!$N$2:$N$42,"="&amp;A5)</f>
-        <v>23</v>
+        <f>COUNTIFS(Respuestas!$N$2:$N$35,"="&amp;A5)</f>
+        <v>20</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>0.56097560975609762</v>
+        <v>0.58823529411764708</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -16246,21 +15767,21 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <f>COUNTIFS(Respuestas!$N$2:$N$42,"="&amp;A6)</f>
-        <v>11</v>
+        <f>COUNTIFS(Respuestas!$N$2:$N$35,"="&amp;A6)</f>
+        <v>7</v>
       </c>
       <c r="C6" s="8">
         <f t="shared" si="0"/>
-        <v>0.26829268292682928</v>
+        <v>0.20588235294117646</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8">
         <f>SUM(C2:C6)</f>

</xml_diff>